<commit_message>
Before big mortality changes
</commit_message>
<xml_diff>
--- a/data/TierPlus Parameter Lists - Shared.xlsx
+++ b/data/TierPlus Parameter Lists - Shared.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="173" documentId="8_{3B20D403-37D7-C947-81A8-DEC9FA14756B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6FA93D1-4D89-4F78-B8AF-CA529289C82A}"/>
+  <xr:revisionPtr revIDLastSave="199" documentId="8_{3B20D403-37D7-C947-81A8-DEC9FA14756B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4486FD15-673D-4171-B1E6-E833B9B35A44}"/>
   <bookViews>
-    <workbookView xWindow="1700" yWindow="500" windowWidth="27020" windowHeight="16100" firstSheet="3" activeTab="2" xr2:uid="{3655CBE5-0E8F-BC41-8085-555297440F15}"/>
+    <workbookView xWindow="1700" yWindow="500" windowWidth="27020" windowHeight="16100" firstSheet="2" activeTab="1" xr2:uid="{3655CBE5-0E8F-BC41-8085-555297440F15}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="7" r:id="rId1"/>
@@ -45,13 +45,37 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Guest User</author>
+    <author>tc={45F02302-2DC4-4212-8298-C9BFF9E71FD2}</author>
   </authors>
   <commentList>
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{750FB328-26C3-43AF-A515-0C539B20F018}">
+      <text>
+        <t>BN: all values to be in USD (and in theory inflated to 2026 USD)</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="1" shapeId="0" xr:uid="{45F02302-2DC4-4212-8298-C9BFF9E71FD2}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    BN:
+Add a link (or links) to the reference(s) for the cost/parameter value </t>
+      </text>
+    </comment>
     <comment ref="G6" authorId="0" shapeId="0" xr:uid="{17498D47-3797-4323-AB1C-C35B26A2CA0B}">
       <text>
-        <t>BN: Tons of data here: 
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color theme="1"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>BN: Tons of data here: 
 https://pubmed.ncbi.nlm.nih.gov/40579870/
 (also in supplement- retention/suppression for each model, and cost of each model).. granted from Zam only</t>
+        </r>
       </text>
     </comment>
   </commentList>
@@ -59,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="731" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="731" uniqueCount="199">
   <si>
     <t>Values need to incoporate realistic implementation and weighted effects</t>
   </si>
@@ -163,13 +187,13 @@
     <t>mmd_6month</t>
   </si>
   <si>
-    <t>Community pharmacy pick-ups</t>
+    <t>DSD: Community pharmacy pick-up</t>
   </si>
   <si>
     <t>DSD_communitypharm</t>
   </si>
   <si>
-    <t>Fast-track pick-ups</t>
+    <t>DSD: fast-track pick-ups</t>
   </si>
   <si>
     <t>DSD_fasttrack</t>
@@ -448,6 +472,9 @@
     <t>Yield multiplier</t>
   </si>
   <si>
+    <t>Going to use country-specific GAM data for this</t>
+  </si>
+  <si>
     <t>Proportion of positive tests that link to ART</t>
   </si>
   <si>
@@ -520,18 +547,30 @@
     <t>description</t>
   </si>
   <si>
+    <t>Notes</t>
+  </si>
+  <si>
     <t>hiv_mortality_suppressed</t>
   </si>
   <si>
     <t>PLACEHOLDER</t>
   </si>
   <si>
+    <t>https://journals.plos.org/plosmedicine/article?id=10.1371/journal.pmed.1000066</t>
+  </si>
+  <si>
     <t>HIV related mortality while indiviudal on treatment and virally suppressed</t>
   </si>
   <si>
+    <t xml:space="preserve">Again, here, maybe something </t>
+  </si>
+  <si>
     <t>hiv_mortality_on_treatment</t>
   </si>
   <si>
+    <t>0.098 (up to 0.63 for AIDS stage... calibration?)</t>
+  </si>
+  <si>
     <t>HIV related mortality while on tretament but not virally suppressed</t>
   </si>
   <si>
@@ -568,7 +607,7 @@
     <t>ltfu_rate</t>
   </si>
   <si>
-    <t>rate of LTFU</t>
+    <t>annual rate of LTFU</t>
   </si>
   <si>
     <t>high_risk_proprtion</t>
@@ -641,19 +680,13 @@
   </si>
   <si>
     <t>Additional MTCT reduction from enhanced PMTCT interventions beyond baseline</t>
-  </si>
-  <si>
-    <t>ART provision cost</t>
-  </si>
-  <si>
-    <t>Annual cost per person on ART (ARVs + service delivery)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -674,8 +707,23 @@
       <name val="Aptos Narrow"/>
       <charset val="1"/>
     </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -694,6 +742,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -704,10 +764,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -715,8 +776,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -730,6 +799,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Guest User" id="{DC91C072-E505-473A-AFFA-5FAA02A1A991}" userId="" providerId="Windows Live"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1047,6 +1122,15 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="G1" dT="2026-03-05T12:33:53.30" personId="{DC91C072-E505-473A-AFFA-5FAA02A1A991}" id="{45F02302-2DC4-4212-8298-C9BFF9E71FD2}">
+    <text xml:space="preserve">BN:
+Add a link (or links) to the reference(s) for the cost/parameter value </text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7895DAEF-CB01-404D-B7FE-91E64BF4FB1F}">
   <dimension ref="A1:A9"/>
@@ -2192,7 +2276,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A7EA96D-7C78-2A4B-AAB8-1FB20EF8C6D6}">
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
   <cols>
     <col min="1" max="1" width="16.5" bestFit="1" customWidth="1"/>
@@ -2202,7 +2286,7 @@
     <col min="8" max="8" width="73.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="4" customFormat="1">
+    <row r="1" spans="1:9" s="4" customFormat="1">
       <c r="A1" s="4" t="s">
         <v>7</v>
       </c>
@@ -2228,7 +2312,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
         <v>47</v>
       </c>
@@ -2254,7 +2338,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
         <v>47</v>
       </c>
@@ -2280,7 +2364,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
         <v>47</v>
       </c>
@@ -2306,7 +2390,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:9">
       <c r="A5" t="s">
         <v>47</v>
       </c>
@@ -2332,7 +2416,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:9">
       <c r="A6" t="s">
         <v>47</v>
       </c>
@@ -2358,7 +2442,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:9">
       <c r="A7" t="s">
         <v>47</v>
       </c>
@@ -2384,553 +2468,576 @@
         <v>122</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
-      <c r="A8" t="s">
-        <v>79</v>
-      </c>
-      <c r="B8" t="s">
+    <row r="8" spans="1:9">
+      <c r="A8" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="7">
         <v>0.97</v>
       </c>
-      <c r="F8" t="s">
-        <v>20</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H8" t="s">
+      <c r="F8" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8" s="7" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="9" spans="1:8">
-      <c r="A9" t="s">
-        <v>79</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="I8" s="8"/>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B9" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="7">
         <v>0.8</v>
       </c>
-      <c r="F9" t="s">
-        <v>20</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H9" t="s">
+      <c r="F9" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H9" s="7" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="A10" t="s">
-        <v>79</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="I9" s="8"/>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="7">
         <v>2</v>
       </c>
-      <c r="F10" t="s">
-        <v>20</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H10" t="s">
+      <c r="F10" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H10" s="7" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" t="s">
-        <v>79</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="I10" s="8"/>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="7">
         <v>0.97</v>
       </c>
-      <c r="F11" t="s">
-        <v>20</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H11" t="s">
+      <c r="F11" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H11" s="7" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="12" spans="1:8">
-      <c r="A12" t="s">
-        <v>79</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="I11" s="8"/>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B12" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="7">
         <v>0.9</v>
       </c>
-      <c r="F12" t="s">
-        <v>20</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H12" t="s">
+      <c r="F12" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H12" s="7" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="13" spans="1:8">
-      <c r="A13" t="s">
-        <v>79</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="I12" s="8"/>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="7">
         <v>1</v>
       </c>
-      <c r="F13" t="s">
-        <v>20</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H13" t="s">
+      <c r="F13" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H13" s="7" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="14" spans="1:8">
-      <c r="A14" t="s">
-        <v>79</v>
-      </c>
-      <c r="B14" t="s">
+      <c r="I13" s="8"/>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="7">
         <v>0.99</v>
       </c>
-      <c r="F14" t="s">
-        <v>20</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H14" t="s">
+      <c r="F14" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H14" s="7" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="15" spans="1:8">
-      <c r="A15" t="s">
-        <v>79</v>
-      </c>
-      <c r="B15" t="s">
+      <c r="I14" s="8"/>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B15" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="7">
         <v>0.97</v>
       </c>
-      <c r="F15" t="s">
-        <v>20</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H15" t="s">
+      <c r="F15" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H15" s="7" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="16" spans="1:8">
-      <c r="A16" t="s">
-        <v>79</v>
-      </c>
-      <c r="B16" t="s">
+      <c r="I15" s="8"/>
+    </row>
+    <row r="16" spans="1:9" ht="77.25">
+      <c r="A16" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B16" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="E16">
+      <c r="E16" s="7">
         <v>1</v>
       </c>
-      <c r="F16" t="s">
-        <v>20</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H16" t="s">
+      <c r="F16" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H16" s="7" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="17" spans="1:8">
-      <c r="A17" t="s">
-        <v>79</v>
-      </c>
-      <c r="B17" t="s">
+      <c r="I16" s="9" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="7">
         <v>0.99</v>
       </c>
-      <c r="F17" t="s">
-        <v>20</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H17" t="s">
+      <c r="F17" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H17" s="7" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="18" spans="1:8">
-      <c r="A18" t="s">
-        <v>79</v>
-      </c>
-      <c r="B18" t="s">
+      <c r="I17" s="8"/>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B18" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="E18">
+      <c r="E18" s="7">
         <v>0.97</v>
       </c>
-      <c r="F18" t="s">
-        <v>20</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H18" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8">
-      <c r="A19" t="s">
-        <v>79</v>
-      </c>
-      <c r="B19" t="s">
+      <c r="F18" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="I18" s="8"/>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B19" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="E19">
+      <c r="E19" s="7">
         <v>1</v>
       </c>
-      <c r="F19" t="s">
-        <v>20</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H19" t="s">
+      <c r="F19" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H19" s="7" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="20" spans="1:8">
-      <c r="A20" t="s">
-        <v>79</v>
-      </c>
-      <c r="B20" t="s">
+      <c r="I19" s="8"/>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B20" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="E20">
+      <c r="E20" s="7">
         <v>0.99</v>
       </c>
-      <c r="F20" t="s">
-        <v>20</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H20" t="s">
+      <c r="F20" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H20" s="7" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="21" spans="1:8">
-      <c r="A21" t="s">
-        <v>79</v>
-      </c>
-      <c r="B21" t="s">
+      <c r="I20" s="8"/>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B21" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="E21">
+      <c r="E21" s="7">
         <v>0.97</v>
       </c>
-      <c r="F21" t="s">
-        <v>20</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H21" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8">
-      <c r="A22" t="s">
-        <v>79</v>
-      </c>
-      <c r="B22" t="s">
+      <c r="F21" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="I21" s="8"/>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B22" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="E22">
+      <c r="E22" s="7">
         <v>1.5</v>
       </c>
-      <c r="F22" t="s">
-        <v>20</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H22" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8">
-      <c r="A23" t="s">
-        <v>79</v>
-      </c>
-      <c r="B23" t="s">
+      <c r="F22" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="I22" s="8"/>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="E23">
+      <c r="E23" s="7">
         <v>0.97</v>
       </c>
-      <c r="F23" t="s">
-        <v>20</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H23" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8">
-      <c r="A24" t="s">
-        <v>79</v>
-      </c>
-      <c r="B24" t="s">
+      <c r="F23" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="I23" s="8"/>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B24" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="E24">
+      <c r="E24" s="7">
         <v>0.7</v>
       </c>
-      <c r="F24" t="s">
-        <v>20</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H24" t="s">
+      <c r="F24" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="I24" s="8"/>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="E25" s="7">
+        <v>1</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="I25" s="8"/>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="E26" s="7">
+        <v>0.97</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H26" s="7" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="25" spans="1:8">
-      <c r="A25" t="s">
-        <v>79</v>
-      </c>
-      <c r="B25" t="s">
-        <v>93</v>
-      </c>
-      <c r="C25" t="s">
-        <v>94</v>
-      </c>
-      <c r="D25" t="s">
+      <c r="I26" s="8"/>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="E27" s="7">
+        <v>0.7</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G27" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H27" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="I27" s="8"/>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="D28" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="E25">
+      <c r="E28" s="7">
         <v>1</v>
       </c>
-      <c r="F25" t="s">
-        <v>20</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H25" t="s">
+      <c r="F28" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H28" s="7" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>79</v>
-      </c>
-      <c r="B26" t="s">
-        <v>89</v>
-      </c>
-      <c r="C26" t="s">
-        <v>90</v>
-      </c>
-      <c r="D26" t="s">
-        <v>115</v>
-      </c>
-      <c r="E26">
-        <v>0.97</v>
-      </c>
-      <c r="F26" t="s">
-        <v>20</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H26" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8">
-      <c r="A27" t="s">
-        <v>79</v>
-      </c>
-      <c r="B27" t="s">
-        <v>89</v>
-      </c>
-      <c r="C27" t="s">
-        <v>90</v>
-      </c>
-      <c r="D27" t="s">
-        <v>124</v>
-      </c>
-      <c r="E27">
-        <v>0.7</v>
-      </c>
-      <c r="F27" t="s">
-        <v>20</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H27" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8">
-      <c r="A28" t="s">
-        <v>79</v>
-      </c>
-      <c r="B28" t="s">
-        <v>89</v>
-      </c>
-      <c r="C28" t="s">
-        <v>90</v>
-      </c>
-      <c r="D28" t="s">
-        <v>126</v>
-      </c>
-      <c r="E28">
-        <v>1</v>
-      </c>
-      <c r="F28" t="s">
-        <v>20</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H28" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8">
+      <c r="I28" s="8"/>
+    </row>
+    <row r="29" spans="1:9">
       <c r="A29" t="s">
         <v>79</v>
       </c>
@@ -2953,10 +3060,10 @@
         <v>21</v>
       </c>
       <c r="H29" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
       <c r="A30" t="s">
         <v>79</v>
       </c>
@@ -2979,10 +3086,10 @@
         <v>21</v>
       </c>
       <c r="H30" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9">
       <c r="A31" t="s">
         <v>79</v>
       </c>
@@ -3008,7 +3115,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="32" spans="1:8">
+    <row r="32" spans="1:9">
       <c r="A32" t="s">
         <v>79</v>
       </c>
@@ -3031,7 +3138,7 @@
         <v>21</v>
       </c>
       <c r="H32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -3057,7 +3164,7 @@
         <v>21</v>
       </c>
       <c r="H33" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -3109,7 +3216,7 @@
         <v>21</v>
       </c>
       <c r="H35" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -3135,7 +3242,7 @@
         <v>21</v>
       </c>
       <c r="H36" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -3181,13 +3288,13 @@
         <v>0.3</v>
       </c>
       <c r="F38" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G38" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H38" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -3213,7 +3320,7 @@
         <v>21</v>
       </c>
       <c r="H39" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -3239,7 +3346,7 @@
         <v>21</v>
       </c>
       <c r="H40" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -3265,7 +3372,7 @@
         <v>21</v>
       </c>
       <c r="H41" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="42" spans="1:8">
@@ -3291,7 +3398,7 @@
         <v>21</v>
       </c>
       <c r="H42" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -3317,7 +3424,7 @@
         <v>21</v>
       </c>
       <c r="H43" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -3343,7 +3450,7 @@
         <v>21</v>
       </c>
       <c r="H44" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -3369,7 +3476,7 @@
         <v>21</v>
       </c>
       <c r="H45" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -3418,7 +3525,7 @@
         <v>21</v>
       </c>
       <c r="H47" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -3428,7 +3535,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6747B679-9230-3847-955E-AE6563A4F4F1}">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
   <cols>
     <col min="1" max="1" width="30" bestFit="1" customWidth="1"/>
@@ -3439,86 +3546,101 @@
     <col min="6" max="6" width="106.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="4" customFormat="1">
+    <row r="1" spans="1:7" s="4" customFormat="1">
       <c r="A1" s="4" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+        <v>153</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15.75">
       <c r="A2" t="s">
-        <v>153</v>
+        <v>155</v>
+      </c>
+      <c r="B2">
+        <v>0.02</v>
       </c>
       <c r="C2" t="s">
-        <v>154</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>21</v>
+        <v>156</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>157</v>
       </c>
       <c r="E2" t="s">
         <v>40</v>
       </c>
       <c r="F2" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>158</v>
+      </c>
+      <c r="G2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="15.75">
       <c r="A3" t="s">
+        <v>160</v>
+      </c>
+      <c r="B3" t="s">
+        <v>161</v>
+      </c>
+      <c r="C3" t="s">
         <v>156</v>
       </c>
-      <c r="C3" t="s">
-        <v>154</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>21</v>
+      <c r="D3" s="10" t="s">
+        <v>157</v>
       </c>
       <c r="E3" t="s">
         <v>40</v>
       </c>
       <c r="F3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="15.75">
+      <c r="A4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C4" t="s">
+        <v>156</v>
+      </c>
+      <c r="D4" s="10" t="s">
         <v>157</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" t="s">
-        <v>158</v>
-      </c>
-      <c r="C4" t="s">
-        <v>154</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>21</v>
       </c>
       <c r="E4" t="s">
         <v>40</v>
       </c>
       <c r="F4" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="B5">
         <v>1.5</v>
       </c>
       <c r="C5" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>21</v>
@@ -3527,18 +3649,18 @@
         <v>40</v>
       </c>
       <c r="F5" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="B6">
         <v>0.6</v>
       </c>
       <c r="C6" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>21</v>
@@ -3547,18 +3669,18 @@
         <v>40</v>
       </c>
       <c r="F6" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="B7">
         <v>0.85</v>
       </c>
       <c r="C7" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>21</v>
@@ -3567,18 +3689,18 @@
         <v>40</v>
       </c>
       <c r="F7" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="B8">
         <v>0.08</v>
       </c>
       <c r="C8" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>21</v>
@@ -3587,18 +3709,18 @@
         <v>40</v>
       </c>
       <c r="F8" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="B9">
         <v>0.15</v>
       </c>
       <c r="C9" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>21</v>
@@ -3607,18 +3729,18 @@
         <v>40</v>
       </c>
       <c r="F9" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="B10">
         <v>0.05</v>
       </c>
       <c r="C10" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>21</v>
@@ -3627,38 +3749,38 @@
         <v>40</v>
       </c>
       <c r="F10" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="B11">
         <v>0.25</v>
       </c>
       <c r="C11" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E11" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="F11" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B12">
         <v>0.02</v>
       </c>
       <c r="C12" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>21</v>
@@ -3667,18 +3789,18 @@
         <v>40</v>
       </c>
       <c r="F12" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="B13">
         <v>0.2</v>
       </c>
       <c r="C13" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>21</v>
@@ -3687,18 +3809,18 @@
         <v>40</v>
       </c>
       <c r="F13" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B14">
         <v>0.9</v>
       </c>
       <c r="C14" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>21</v>
@@ -3707,18 +3829,18 @@
         <v>40</v>
       </c>
       <c r="F14" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="B15">
         <v>0.9</v>
       </c>
       <c r="C15" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>21</v>
@@ -3727,18 +3849,18 @@
         <v>40</v>
       </c>
       <c r="F15" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="B16">
         <v>0.1</v>
       </c>
       <c r="C16" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>21</v>
@@ -3747,52 +3869,52 @@
         <v>40</v>
       </c>
       <c r="F16" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="B17">
         <v>0.5</v>
       </c>
       <c r="C17" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E17" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="F17" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="1" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="B18" s="1">
         <v>0.9</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>21</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="B19">
         <v>0.15</v>
@@ -3804,15 +3926,15 @@
         <v>21</v>
       </c>
       <c r="E19" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="F19" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="B20">
         <v>0.3</v>
@@ -3827,30 +3949,23 @@
         <v>40</v>
       </c>
       <c r="F20" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
     </row>
     <row r="21" spans="1:6">
-      <c r="A21" t="s">
-        <v>194</v>
-      </c>
-      <c r="B21">
-        <v>200</v>
-      </c>
-      <c r="C21" t="s">
-        <v>20</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E21" t="s">
-        <v>40</v>
-      </c>
-      <c r="F21" t="s">
-        <v>195</v>
-      </c>
+      <c r="A21" s="11"/>
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{6B6708C6-EB81-454F-A9C6-9626501069D8}"/>
+    <hyperlink ref="D3" r:id="rId2" xr:uid="{7BE220D3-85E1-4DB4-98CC-979C5E6EC84C}"/>
+    <hyperlink ref="D4" r:id="rId3" xr:uid="{848487C8-1AFC-4EF1-832E-CAB730114204}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
First retention changes - unchecked
</commit_message>
<xml_diff>
--- a/data/TierPlus Parameter Lists - Shared.xlsx
+++ b/data/TierPlus Parameter Lists - Shared.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29825"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29905"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="199" documentId="8_{3B20D403-37D7-C947-81A8-DEC9FA14756B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4486FD15-673D-4171-B1E6-E833B9B35A44}"/>
+  <xr:revisionPtr revIDLastSave="200" documentId="8_{3B20D403-37D7-C947-81A8-DEC9FA14756B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{218C5C5F-F21A-4AE2-B8DF-69CC56D4693F}"/>
   <bookViews>
-    <workbookView xWindow="1700" yWindow="500" windowWidth="27020" windowHeight="16100" firstSheet="2" activeTab="1" xr2:uid="{3655CBE5-0E8F-BC41-8085-555297440F15}"/>
+    <workbookView xWindow="1700" yWindow="500" windowWidth="27020" windowHeight="16100" firstSheet="1" activeTab="1" xr2:uid="{3655CBE5-0E8F-BC41-8085-555297440F15}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="7" r:id="rId1"/>
@@ -50,7 +50,16 @@
   <commentList>
     <comment ref="E1" authorId="0" shapeId="0" xr:uid="{750FB328-26C3-43AF-A515-0C539B20F018}">
       <text>
-        <t>BN: all values to be in USD (and in theory inflated to 2026 USD)</t>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color theme="1"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>BN: all values to be in USD (and in theory inflated to 2026 USD)</t>
+        </r>
       </text>
     </comment>
     <comment ref="G1" authorId="1" shapeId="0" xr:uid="{45F02302-2DC4-4212-8298-C9BFF9E71FD2}">
@@ -83,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="731" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="731" uniqueCount="200">
   <si>
     <t>Values need to incoporate realistic implementation and weighted effects</t>
   </si>
@@ -185,6 +194,9 @@
   </si>
   <si>
     <t>mmd_6month</t>
+  </si>
+  <si>
+    <t>Is</t>
   </si>
   <si>
     <t>DSD: Community pharmacy pick-up</t>
@@ -1350,7 +1362,7 @@
         <v>21</v>
       </c>
       <c r="H6" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -1358,10 +1370,10 @@
         <v>26</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D7" t="s">
         <v>19</v>
@@ -1384,10 +1396,10 @@
         <v>26</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D8" t="s">
         <v>19</v>
@@ -1407,13 +1419,13 @@
     </row>
     <row r="9" spans="1:9">
       <c r="A9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D9" t="s">
         <v>19</v>
@@ -1436,10 +1448,10 @@
         <v>26</v>
       </c>
       <c r="B10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D10" t="s">
         <v>19</v>
@@ -1454,7 +1466,7 @@
         <v>21</v>
       </c>
       <c r="H10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -1462,10 +1474,10 @@
         <v>26</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D11" t="s">
         <v>19</v>
@@ -1480,18 +1492,18 @@
         <v>21</v>
       </c>
       <c r="H11" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12" spans="1:9">
       <c r="A12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D12" t="s">
         <v>19</v>
@@ -1506,18 +1518,18 @@
         <v>21</v>
       </c>
       <c r="H12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:9">
       <c r="A13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C13" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D13" t="s">
         <v>19</v>
@@ -1532,18 +1544,18 @@
         <v>21</v>
       </c>
       <c r="H13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14" spans="1:9">
       <c r="A14" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D14" t="s">
         <v>19</v>
@@ -1558,18 +1570,18 @@
         <v>21</v>
       </c>
       <c r="H14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B15" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C15" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D15" t="s">
         <v>19</v>
@@ -1584,18 +1596,18 @@
         <v>21</v>
       </c>
       <c r="H15" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:9">
       <c r="A16" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B16" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C16" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D16" t="s">
         <v>19</v>
@@ -1610,18 +1622,18 @@
         <v>21</v>
       </c>
       <c r="H16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B17" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C17" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D17" t="s">
         <v>19</v>
@@ -1636,18 +1648,18 @@
         <v>21</v>
       </c>
       <c r="H17" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B18" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C18" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D18" t="s">
         <v>19</v>
@@ -1662,18 +1674,18 @@
         <v>21</v>
       </c>
       <c r="H18" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B19" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C19" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D19" t="s">
         <v>19</v>
@@ -1688,18 +1700,18 @@
         <v>21</v>
       </c>
       <c r="H19" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20" spans="1:8">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B20" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C20" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D20" t="s">
         <v>19</v>
@@ -1714,18 +1726,18 @@
         <v>21</v>
       </c>
       <c r="H20" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B21" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C21" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D21" t="s">
         <v>19</v>
@@ -1740,18 +1752,18 @@
         <v>21</v>
       </c>
       <c r="H21" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="22" spans="1:8">
       <c r="A22" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B22" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C22" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D22" t="s">
         <v>19</v>
@@ -1766,21 +1778,21 @@
         <v>21</v>
       </c>
       <c r="H22" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="23" spans="1:8">
       <c r="A23" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B23" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C23" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D23" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E23">
         <v>4</v>
@@ -1792,18 +1804,18 @@
         <v>21</v>
       </c>
       <c r="H23" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="24" spans="1:8">
       <c r="A24" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B24" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D24" t="s">
         <v>19</v>
@@ -1818,21 +1830,21 @@
         <v>21</v>
       </c>
       <c r="H24" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="25" spans="1:8">
       <c r="A25" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B25" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D25" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E25">
         <v>10</v>
@@ -1844,18 +1856,18 @@
         <v>21</v>
       </c>
       <c r="H25" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="26" spans="1:8">
       <c r="A26" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B26" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C26" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D26" t="s">
         <v>19</v>
@@ -1870,21 +1882,21 @@
         <v>21</v>
       </c>
       <c r="H26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="27" spans="1:8">
       <c r="A27" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B27" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C27" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D27" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E27">
         <v>0</v>
@@ -1896,18 +1908,18 @@
         <v>21</v>
       </c>
       <c r="H27" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="15.75">
       <c r="A28" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B28" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C28" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D28" t="s">
         <v>19</v>
@@ -1922,21 +1934,21 @@
         <v>21</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="29" spans="1:8">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B29" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C29" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D29" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E29">
         <v>0</v>
@@ -1948,18 +1960,18 @@
         <v>21</v>
       </c>
       <c r="H29" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="30" spans="1:8">
       <c r="A30" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B30" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C30" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D30" t="s">
         <v>19</v>
@@ -1974,21 +1986,21 @@
         <v>21</v>
       </c>
       <c r="H30" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="31" spans="1:8">
       <c r="A31" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B31" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C31" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D31" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E31">
         <v>2</v>
@@ -2000,18 +2012,18 @@
         <v>21</v>
       </c>
       <c r="H31" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="32" spans="1:8">
       <c r="A32" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B32" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C32" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D32" t="s">
         <v>19</v>
@@ -2026,21 +2038,21 @@
         <v>21</v>
       </c>
       <c r="H32" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="33" spans="1:8">
       <c r="A33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B33" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C33" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D33" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E33">
         <v>2</v>
@@ -2052,18 +2064,18 @@
         <v>21</v>
       </c>
       <c r="H33" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="34" spans="1:8">
       <c r="A34" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B34" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C34" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D34" t="s">
         <v>19</v>
@@ -2078,21 +2090,21 @@
         <v>21</v>
       </c>
       <c r="H34" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="35" spans="1:8">
       <c r="A35" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B35" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C35" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D35" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E35">
         <v>1</v>
@@ -2104,18 +2116,18 @@
         <v>21</v>
       </c>
       <c r="H35" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="36" spans="1:8">
       <c r="A36" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B36" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C36" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D36" t="s">
         <v>19</v>
@@ -2130,21 +2142,21 @@
         <v>21</v>
       </c>
       <c r="H36" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="37" spans="1:8">
       <c r="A37" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B37" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C37" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D37" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E37">
         <v>1</v>
@@ -2156,18 +2168,18 @@
         <v>21</v>
       </c>
       <c r="H37" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="38" spans="1:8">
       <c r="A38" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B38" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C38" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D38" t="s">
         <v>19</v>
@@ -2182,21 +2194,21 @@
         <v>21</v>
       </c>
       <c r="H38" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="39" spans="1:8">
       <c r="A39" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B39" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C39" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D39" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E39">
         <v>2</v>
@@ -2208,18 +2220,18 @@
         <v>21</v>
       </c>
       <c r="H39" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="40" spans="1:8">
       <c r="A40" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B40" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C40" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D40" t="s">
         <v>19</v>
@@ -2234,21 +2246,21 @@
         <v>21</v>
       </c>
       <c r="H40" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="41" spans="1:8">
       <c r="A41" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B41" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C41" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D41" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E41">
         <v>4</v>
@@ -2260,7 +2272,7 @@
         <v>21</v>
       </c>
       <c r="H41" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -2314,42 +2326,42 @@
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E2">
         <v>0.86</v>
       </c>
       <c r="F2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E3">
         <v>0.96</v>
@@ -2361,21 +2373,21 @@
         <v>21</v>
       </c>
       <c r="H3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D4" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E4">
         <v>0.85</v>
@@ -2387,21 +2399,21 @@
         <v>21</v>
       </c>
       <c r="H4" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E5">
         <v>0.81</v>
@@ -2413,21 +2425,21 @@
         <v>21</v>
       </c>
       <c r="H5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E6">
         <v>0.92</v>
@@ -2439,21 +2451,21 @@
         <v>21</v>
       </c>
       <c r="H6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E7">
         <v>0.7</v>
@@ -2465,21 +2477,21 @@
         <v>21</v>
       </c>
       <c r="H7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E8" s="7">
         <v>0.97</v>
@@ -2491,22 +2503,22 @@
         <v>21</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I8" s="8"/>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E9" s="7">
         <v>0.8</v>
@@ -2518,22 +2530,22 @@
         <v>21</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="I9" s="8"/>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E10" s="7">
         <v>2</v>
@@ -2545,22 +2557,22 @@
         <v>21</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="I10" s="8"/>
     </row>
     <row r="11" spans="1:9">
       <c r="A11" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E11" s="7">
         <v>0.97</v>
@@ -2572,22 +2584,22 @@
         <v>21</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I11" s="8"/>
     </row>
     <row r="12" spans="1:9">
       <c r="A12" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E12" s="7">
         <v>0.9</v>
@@ -2599,22 +2611,22 @@
         <v>21</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="I12" s="8"/>
     </row>
     <row r="13" spans="1:9">
       <c r="A13" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E13" s="7">
         <v>1</v>
@@ -2626,22 +2638,22 @@
         <v>21</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="I13" s="8"/>
     </row>
     <row r="14" spans="1:9">
       <c r="A14" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E14" s="7">
         <v>0.99</v>
@@ -2653,22 +2665,22 @@
         <v>21</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I14" s="8"/>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E15" s="7">
         <v>0.97</v>
@@ -2680,22 +2692,22 @@
         <v>21</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="I15" s="8"/>
     </row>
     <row r="16" spans="1:9" ht="77.25">
       <c r="A16" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E16" s="7">
         <v>1</v>
@@ -2707,24 +2719,24 @@
         <v>21</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="I16" s="9" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E17" s="7">
         <v>0.99</v>
@@ -2736,22 +2748,22 @@
         <v>21</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I17" s="8"/>
     </row>
     <row r="18" spans="1:9">
       <c r="A18" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E18" s="7">
         <v>0.97</v>
@@ -2763,22 +2775,22 @@
         <v>21</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I18" s="8"/>
     </row>
     <row r="19" spans="1:9">
       <c r="A19" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E19" s="7">
         <v>1</v>
@@ -2790,22 +2802,22 @@
         <v>21</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="I19" s="8"/>
     </row>
     <row r="20" spans="1:9">
       <c r="A20" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E20" s="7">
         <v>0.99</v>
@@ -2817,22 +2829,22 @@
         <v>21</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I20" s="8"/>
     </row>
     <row r="21" spans="1:9">
       <c r="A21" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E21" s="7">
         <v>0.97</v>
@@ -2844,22 +2856,22 @@
         <v>21</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I21" s="8"/>
     </row>
     <row r="22" spans="1:9">
       <c r="A22" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E22" s="7">
         <v>1.5</v>
@@ -2871,22 +2883,22 @@
         <v>21</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="I22" s="8"/>
     </row>
     <row r="23" spans="1:9">
       <c r="A23" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E23" s="7">
         <v>0.97</v>
@@ -2898,22 +2910,22 @@
         <v>21</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I23" s="8"/>
     </row>
     <row r="24" spans="1:9">
       <c r="A24" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E24" s="7">
         <v>0.7</v>
@@ -2925,22 +2937,22 @@
         <v>21</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I24" s="8"/>
     </row>
     <row r="25" spans="1:9">
       <c r="A25" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E25" s="7">
         <v>1</v>
@@ -2952,22 +2964,22 @@
         <v>21</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="I25" s="8"/>
     </row>
     <row r="26" spans="1:9">
       <c r="A26" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E26" s="7">
         <v>0.97</v>
@@ -2979,22 +2991,22 @@
         <v>21</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I26" s="8"/>
     </row>
     <row r="27" spans="1:9">
       <c r="A27" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E27" s="7">
         <v>0.7</v>
@@ -3006,22 +3018,22 @@
         <v>21</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I27" s="8"/>
     </row>
     <row r="28" spans="1:9">
       <c r="A28" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E28" s="7">
         <v>1</v>
@@ -3033,22 +3045,22 @@
         <v>21</v>
       </c>
       <c r="H28" s="7" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="I28" s="8"/>
     </row>
     <row r="29" spans="1:9">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B29" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C29" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D29" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E29">
         <v>0.98</v>
@@ -3060,21 +3072,21 @@
         <v>21</v>
       </c>
       <c r="H29" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="30" spans="1:9">
       <c r="A30" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B30" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C30" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D30" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E30">
         <v>0.95</v>
@@ -3086,21 +3098,21 @@
         <v>21</v>
       </c>
       <c r="H30" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="31" spans="1:9">
       <c r="A31" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B31" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C31" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D31" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -3112,21 +3124,21 @@
         <v>21</v>
       </c>
       <c r="H31" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="32" spans="1:9">
       <c r="A32" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B32" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C32" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D32" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E32">
         <v>0.99</v>
@@ -3138,21 +3150,21 @@
         <v>21</v>
       </c>
       <c r="H32" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="33" spans="1:8">
       <c r="A33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B33" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C33" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D33" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E33">
         <v>0.97</v>
@@ -3164,21 +3176,21 @@
         <v>21</v>
       </c>
       <c r="H33" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="34" spans="1:8">
       <c r="A34" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B34" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C34" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D34" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E34">
         <v>1</v>
@@ -3190,21 +3202,21 @@
         <v>21</v>
       </c>
       <c r="H34" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="35" spans="1:8">
       <c r="A35" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B35" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C35" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D35" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E35">
         <v>0.99</v>
@@ -3216,21 +3228,21 @@
         <v>21</v>
       </c>
       <c r="H35" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="36" spans="1:8">
       <c r="A36" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B36" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C36" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D36" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E36">
         <v>0.97</v>
@@ -3242,21 +3254,21 @@
         <v>21</v>
       </c>
       <c r="H36" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="37" spans="1:8">
       <c r="A37" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B37" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C37" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D37" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E37">
         <v>1</v>
@@ -3268,7 +3280,7 @@
         <v>21</v>
       </c>
       <c r="H37" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -3276,25 +3288,25 @@
         <v>26</v>
       </c>
       <c r="B38" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C38" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D38" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E38">
         <v>0.3</v>
       </c>
       <c r="F38" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G38" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H38" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -3302,13 +3314,13 @@
         <v>26</v>
       </c>
       <c r="B39" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D39" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E39">
         <v>0.75</v>
@@ -3320,7 +3332,7 @@
         <v>21</v>
       </c>
       <c r="H39" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -3334,7 +3346,7 @@
         <v>31</v>
       </c>
       <c r="D40" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E40">
         <v>0.88</v>
@@ -3346,7 +3358,7 @@
         <v>21</v>
       </c>
       <c r="H40" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -3360,7 +3372,7 @@
         <v>33</v>
       </c>
       <c r="D41" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E41">
         <v>0.92</v>
@@ -3372,7 +3384,7 @@
         <v>21</v>
       </c>
       <c r="H41" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="42" spans="1:8">
@@ -3386,7 +3398,7 @@
         <v>28</v>
       </c>
       <c r="D42" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E42">
         <v>0.95</v>
@@ -3398,21 +3410,21 @@
         <v>21</v>
       </c>
       <c r="H42" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="43" spans="1:8">
       <c r="A43" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B43" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C43" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D43" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E43">
         <v>0.8</v>
@@ -3424,21 +3436,21 @@
         <v>21</v>
       </c>
       <c r="H43" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="44" spans="1:8">
       <c r="A44" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B44" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C44" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D44" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E44">
         <v>0.3</v>
@@ -3450,21 +3462,21 @@
         <v>21</v>
       </c>
       <c r="H44" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="45" spans="1:8">
       <c r="A45" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B45" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C45" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D45" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E45">
         <v>0.88</v>
@@ -3476,7 +3488,7 @@
         <v>21</v>
       </c>
       <c r="H45" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -3490,7 +3502,7 @@
         <v>24</v>
       </c>
       <c r="D46" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E46">
         <v>1</v>
@@ -3513,7 +3525,7 @@
         <v>18</v>
       </c>
       <c r="D47" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E47">
         <v>0.85</v>
@@ -3525,7 +3537,7 @@
         <v>21</v>
       </c>
       <c r="H47" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -3548,373 +3560,373 @@
   <sheetData>
     <row r="1" spans="1:7" s="4" customFormat="1">
       <c r="A1" s="4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="15.75">
       <c r="A2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B2">
         <v>0.02</v>
       </c>
       <c r="C2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="15.75">
       <c r="A3" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C3" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="15.75">
       <c r="A4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C4" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F4" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B5">
         <v>1.5</v>
       </c>
       <c r="C5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B6">
         <v>0.6</v>
       </c>
       <c r="C6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B7">
         <v>0.85</v>
       </c>
       <c r="C7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F7" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B8">
         <v>0.08</v>
       </c>
       <c r="C8" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B9">
         <v>0.15</v>
       </c>
       <c r="C9" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B10">
         <v>0.05</v>
       </c>
       <c r="C10" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E10" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B11">
         <v>0.25</v>
       </c>
       <c r="C11" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E11" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F11" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B12">
         <v>0.02</v>
       </c>
       <c r="C12" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F12" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B13">
         <v>0.2</v>
       </c>
       <c r="C13" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E13" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F13" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B14">
         <v>0.9</v>
       </c>
       <c r="C14" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E14" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B15">
         <v>0.9</v>
       </c>
       <c r="C15" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E15" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F15" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B16">
         <v>0.1</v>
       </c>
       <c r="C16" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E16" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F16" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B17">
         <v>0.5</v>
       </c>
       <c r="C17" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E17" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F17" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B18" s="1">
         <v>0.9</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>21</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B19">
         <v>0.15</v>
@@ -3926,15 +3938,15 @@
         <v>21</v>
       </c>
       <c r="E19" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F19" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B20">
         <v>0.3</v>
@@ -3946,10 +3958,10 @@
         <v>21</v>
       </c>
       <c r="E20" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F20" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="21" spans="1:6">

</xml_diff>

<commit_message>
HTS Testing summary data
</commit_message>
<xml_diff>
--- a/data/TierPlus Parameter Lists - Shared.xlsx
+++ b/data/TierPlus Parameter Lists - Shared.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29910"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="210" documentId="8_{3B20D403-37D7-C947-81A8-DEC9FA14756B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7E88B48-33E0-834B-8CE2-707805D3591D}"/>
+  <xr:revisionPtr revIDLastSave="215" documentId="8_{3B20D403-37D7-C947-81A8-DEC9FA14756B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C8DCF936-BE31-4918-809D-F0B1E73DFD8F}"/>
   <bookViews>
-    <workbookView xWindow="1700" yWindow="600" windowWidth="27020" windowHeight="15820" firstSheet="1" activeTab="3" xr2:uid="{3655CBE5-0E8F-BC41-8085-555297440F15}"/>
+    <workbookView xWindow="1700" yWindow="600" windowWidth="27020" windowHeight="15820" firstSheet="3" xr2:uid="{3655CBE5-0E8F-BC41-8085-555297440F15}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="7" r:id="rId1"/>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="745" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="745" uniqueCount="201">
   <si>
     <t>Values need to incoporate realistic implementation and weighted effects</t>
   </si>
@@ -196,9 +196,6 @@
     <t>mmd_6month</t>
   </si>
   <si>
-    <t>Is</t>
-  </si>
-  <si>
     <t>DSD: Community pharmacy pick-up</t>
   </si>
   <si>
@@ -541,6 +538,12 @@
     <t>Mortality reduction from full AHD package (LAM + CrAg + fluconazole)</t>
   </si>
   <si>
+    <t>Retention improvement vs clinic dispensing</t>
+  </si>
+  <si>
+    <t>Retention improvement vs standard clinic visit</t>
+  </si>
+  <si>
     <t>variable</t>
   </si>
   <si>
@@ -692,19 +695,13 @@
   </si>
   <si>
     <t>Additional MTCT reduction from enhanced PMTCT interventions beyond baseline</t>
-  </si>
-  <si>
-    <t>Retention improvement vs clinic dispensing</t>
-  </si>
-  <si>
-    <t>Retention improvement vs standard clinic visit</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1148,42 +1145,42 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7895DAEF-CB01-404D-B7FE-91E64BF4FB1F}">
   <dimension ref="A1:A9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
   <cols>
-    <col min="1" max="1" width="90.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="90.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:1">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:1">
       <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:1">
       <c r="A5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:1">
       <c r="A7" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:1">
       <c r="A8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:1">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -1196,19 +1193,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72C465B1-0BF9-9244-AFCE-CE4E419AA7EF}">
   <dimension ref="A1:I41"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
   <cols>
     <col min="1" max="1" width="16.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="27.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="57.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="57.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" s="3" customFormat="1">
       <c r="A1" s="3" t="s">
         <v>7</v>
       </c>
@@ -1237,7 +1234,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -1263,7 +1260,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -1289,7 +1286,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -1315,7 +1312,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9">
       <c r="A5" t="s">
         <v>26</v>
       </c>
@@ -1341,7 +1338,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9">
       <c r="A6" t="s">
         <v>26</v>
       </c>
@@ -1364,18 +1361,18 @@
         <v>21</v>
       </c>
       <c r="H6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
       <c r="A7" t="s">
         <v>26</v>
       </c>
       <c r="B7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" t="s">
         <v>35</v>
-      </c>
-      <c r="C7" t="s">
-        <v>36</v>
       </c>
       <c r="D7" t="s">
         <v>19</v>
@@ -1393,15 +1390,15 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9">
       <c r="A8" t="s">
         <v>26</v>
       </c>
       <c r="B8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" t="s">
         <v>37</v>
-      </c>
-      <c r="C8" t="s">
-        <v>38</v>
       </c>
       <c r="D8" t="s">
         <v>19</v>
@@ -1419,15 +1416,15 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9">
       <c r="A9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" t="s">
         <v>39</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>40</v>
-      </c>
-      <c r="C9" t="s">
-        <v>41</v>
       </c>
       <c r="D9" t="s">
         <v>19</v>
@@ -1445,15 +1442,15 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9">
       <c r="A10" t="s">
         <v>26</v>
       </c>
       <c r="B10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" t="s">
         <v>42</v>
-      </c>
-      <c r="C10" t="s">
-        <v>43</v>
       </c>
       <c r="D10" t="s">
         <v>19</v>
@@ -1468,18 +1465,18 @@
         <v>21</v>
       </c>
       <c r="H10" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
       <c r="A11" t="s">
         <v>26</v>
       </c>
       <c r="B11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" t="s">
         <v>45</v>
-      </c>
-      <c r="C11" t="s">
-        <v>46</v>
       </c>
       <c r="D11" t="s">
         <v>19</v>
@@ -1494,18 +1491,18 @@
         <v>21</v>
       </c>
       <c r="H11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+      <c r="B12" t="s">
         <v>48</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>49</v>
-      </c>
-      <c r="C12" t="s">
-        <v>50</v>
       </c>
       <c r="D12" t="s">
         <v>19</v>
@@ -1520,18 +1517,18 @@
         <v>21</v>
       </c>
       <c r="H12" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" t="s">
+        <v>47</v>
+      </c>
+      <c r="B13" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>48</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>52</v>
-      </c>
-      <c r="C13" t="s">
-        <v>53</v>
       </c>
       <c r="D13" t="s">
         <v>19</v>
@@ -1546,18 +1543,18 @@
         <v>21</v>
       </c>
       <c r="H13" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>48</v>
-      </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>55</v>
-      </c>
-      <c r="C14" t="s">
-        <v>56</v>
       </c>
       <c r="D14" t="s">
         <v>19</v>
@@ -1572,18 +1569,18 @@
         <v>21</v>
       </c>
       <c r="H14" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" t="s">
+        <v>47</v>
+      </c>
+      <c r="B15" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>58</v>
-      </c>
-      <c r="C15" t="s">
-        <v>59</v>
       </c>
       <c r="D15" t="s">
         <v>19</v>
@@ -1598,18 +1595,18 @@
         <v>21</v>
       </c>
       <c r="H15" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>48</v>
-      </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>61</v>
-      </c>
-      <c r="C16" t="s">
-        <v>62</v>
       </c>
       <c r="D16" t="s">
         <v>19</v>
@@ -1624,18 +1621,18 @@
         <v>21</v>
       </c>
       <c r="H16" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" t="s">
+        <v>47</v>
+      </c>
+      <c r="B17" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>48</v>
-      </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>64</v>
-      </c>
-      <c r="C17" t="s">
-        <v>65</v>
       </c>
       <c r="D17" t="s">
         <v>19</v>
@@ -1650,18 +1647,18 @@
         <v>21</v>
       </c>
       <c r="H17" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>48</v>
-      </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>67</v>
-      </c>
-      <c r="C18" t="s">
-        <v>68</v>
       </c>
       <c r="D18" t="s">
         <v>19</v>
@@ -1676,18 +1673,18 @@
         <v>21</v>
       </c>
       <c r="H18" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+      <c r="B19" t="s">
         <v>70</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>71</v>
-      </c>
-      <c r="C19" t="s">
-        <v>72</v>
       </c>
       <c r="D19" t="s">
         <v>19</v>
@@ -1702,18 +1699,18 @@
         <v>21</v>
       </c>
       <c r="H19" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" t="s">
+        <v>69</v>
+      </c>
+      <c r="B20" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>70</v>
-      </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>74</v>
-      </c>
-      <c r="C20" t="s">
-        <v>75</v>
       </c>
       <c r="D20" t="s">
         <v>19</v>
@@ -1728,18 +1725,18 @@
         <v>21</v>
       </c>
       <c r="H20" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
+      <c r="A21" t="s">
+        <v>69</v>
+      </c>
+      <c r="B21" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>70</v>
-      </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>77</v>
-      </c>
-      <c r="C21" t="s">
-        <v>78</v>
       </c>
       <c r="D21" t="s">
         <v>19</v>
@@ -1754,18 +1751,18 @@
         <v>21</v>
       </c>
       <c r="H21" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
       <c r="A22" t="s">
+        <v>79</v>
+      </c>
+      <c r="B22" t="s">
         <v>80</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
         <v>81</v>
-      </c>
-      <c r="C22" t="s">
-        <v>82</v>
       </c>
       <c r="D22" t="s">
         <v>19</v>
@@ -1780,21 +1777,21 @@
         <v>21</v>
       </c>
       <c r="H22" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" t="s">
+        <v>80</v>
+      </c>
+      <c r="C23" t="s">
+        <v>81</v>
+      </c>
+      <c r="D23" t="s">
         <v>83</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>80</v>
-      </c>
-      <c r="B23" t="s">
-        <v>81</v>
-      </c>
-      <c r="C23" t="s">
-        <v>82</v>
-      </c>
-      <c r="D23" t="s">
-        <v>84</v>
       </c>
       <c r="E23">
         <v>4</v>
@@ -1806,18 +1803,18 @@
         <v>21</v>
       </c>
       <c r="H23" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24" t="s">
+        <v>79</v>
+      </c>
+      <c r="B24" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>80</v>
-      </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>86</v>
-      </c>
-      <c r="C24" t="s">
-        <v>87</v>
       </c>
       <c r="D24" t="s">
         <v>19</v>
@@ -1832,21 +1829,21 @@
         <v>21</v>
       </c>
       <c r="H24" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
       <c r="A25" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B25" t="s">
+        <v>85</v>
+      </c>
+      <c r="C25" t="s">
         <v>86</v>
       </c>
-      <c r="C25" t="s">
-        <v>87</v>
-      </c>
       <c r="D25" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E25">
         <v>10</v>
@@ -1858,18 +1855,18 @@
         <v>21</v>
       </c>
       <c r="H25" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26" t="s">
+        <v>79</v>
+      </c>
+      <c r="B26" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
-        <v>80</v>
-      </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
         <v>90</v>
-      </c>
-      <c r="C26" t="s">
-        <v>91</v>
       </c>
       <c r="D26" t="s">
         <v>19</v>
@@ -1884,21 +1881,21 @@
         <v>21</v>
       </c>
       <c r="H26" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
       <c r="A27" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B27" t="s">
+        <v>89</v>
+      </c>
+      <c r="C27" t="s">
         <v>90</v>
       </c>
-      <c r="C27" t="s">
-        <v>91</v>
-      </c>
       <c r="D27" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E27">
         <v>0</v>
@@ -1910,18 +1907,18 @@
         <v>21</v>
       </c>
       <c r="H27" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
+      <c r="A28" t="s">
+        <v>79</v>
+      </c>
+      <c r="B28" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
-        <v>80</v>
-      </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
         <v>94</v>
-      </c>
-      <c r="C28" t="s">
-        <v>95</v>
       </c>
       <c r="D28" t="s">
         <v>19</v>
@@ -1936,21 +1933,21 @@
         <v>21</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
       <c r="A29" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B29" t="s">
+        <v>93</v>
+      </c>
+      <c r="C29" t="s">
         <v>94</v>
       </c>
-      <c r="C29" t="s">
-        <v>95</v>
-      </c>
       <c r="D29" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E29">
         <v>0</v>
@@ -1962,18 +1959,18 @@
         <v>21</v>
       </c>
       <c r="H29" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B30" t="s">
+        <v>95</v>
+      </c>
+      <c r="C30" t="s">
         <v>96</v>
-      </c>
-      <c r="C30" t="s">
-        <v>97</v>
       </c>
       <c r="D30" t="s">
         <v>19</v>
@@ -1988,21 +1985,21 @@
         <v>21</v>
       </c>
       <c r="H30" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
       <c r="A31" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B31" t="s">
+        <v>95</v>
+      </c>
+      <c r="C31" t="s">
         <v>96</v>
       </c>
-      <c r="C31" t="s">
-        <v>97</v>
-      </c>
       <c r="D31" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E31">
         <v>2</v>
@@ -2014,18 +2011,18 @@
         <v>21</v>
       </c>
       <c r="H31" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
+      <c r="A32" t="s">
+        <v>79</v>
+      </c>
+      <c r="B32" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
-        <v>80</v>
-      </c>
-      <c r="B32" t="s">
+      <c r="C32" t="s">
         <v>100</v>
-      </c>
-      <c r="C32" t="s">
-        <v>101</v>
       </c>
       <c r="D32" t="s">
         <v>19</v>
@@ -2040,21 +2037,21 @@
         <v>21</v>
       </c>
       <c r="H32" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
       <c r="A33" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B33" t="s">
+        <v>99</v>
+      </c>
+      <c r="C33" t="s">
         <v>100</v>
       </c>
-      <c r="C33" t="s">
-        <v>101</v>
-      </c>
       <c r="D33" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E33">
         <v>2</v>
@@ -2066,18 +2063,18 @@
         <v>21</v>
       </c>
       <c r="H33" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
+      <c r="A34" t="s">
+        <v>79</v>
+      </c>
+      <c r="B34" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
-        <v>80</v>
-      </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
         <v>104</v>
-      </c>
-      <c r="C34" t="s">
-        <v>105</v>
       </c>
       <c r="D34" t="s">
         <v>19</v>
@@ -2092,21 +2089,21 @@
         <v>21</v>
       </c>
       <c r="H34" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
       <c r="A35" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B35" t="s">
+        <v>103</v>
+      </c>
+      <c r="C35" t="s">
         <v>104</v>
       </c>
-      <c r="C35" t="s">
-        <v>105</v>
-      </c>
       <c r="D35" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E35">
         <v>1</v>
@@ -2118,18 +2115,18 @@
         <v>21</v>
       </c>
       <c r="H35" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
+      <c r="A36" t="s">
+        <v>79</v>
+      </c>
+      <c r="B36" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>80</v>
-      </c>
-      <c r="B36" t="s">
+      <c r="C36" t="s">
         <v>108</v>
-      </c>
-      <c r="C36" t="s">
-        <v>109</v>
       </c>
       <c r="D36" t="s">
         <v>19</v>
@@ -2144,21 +2141,21 @@
         <v>21</v>
       </c>
       <c r="H36" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
       <c r="A37" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B37" t="s">
+        <v>107</v>
+      </c>
+      <c r="C37" t="s">
         <v>108</v>
       </c>
-      <c r="C37" t="s">
-        <v>109</v>
-      </c>
       <c r="D37" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E37">
         <v>1</v>
@@ -2170,18 +2167,18 @@
         <v>21</v>
       </c>
       <c r="H37" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
       <c r="A38" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B38" t="s">
+        <v>109</v>
+      </c>
+      <c r="C38" t="s">
         <v>110</v>
-      </c>
-      <c r="C38" t="s">
-        <v>111</v>
       </c>
       <c r="D38" t="s">
         <v>19</v>
@@ -2196,21 +2193,21 @@
         <v>21</v>
       </c>
       <c r="H38" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
       <c r="A39" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B39" t="s">
+        <v>109</v>
+      </c>
+      <c r="C39" t="s">
         <v>110</v>
       </c>
-      <c r="C39" t="s">
-        <v>111</v>
-      </c>
       <c r="D39" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E39">
         <v>2</v>
@@ -2222,18 +2219,18 @@
         <v>21</v>
       </c>
       <c r="H39" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
+      <c r="A40" t="s">
+        <v>79</v>
+      </c>
+      <c r="B40" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
-        <v>80</v>
-      </c>
-      <c r="B40" t="s">
+      <c r="C40" t="s">
         <v>114</v>
-      </c>
-      <c r="C40" t="s">
-        <v>115</v>
       </c>
       <c r="D40" t="s">
         <v>19</v>
@@ -2248,21 +2245,21 @@
         <v>21</v>
       </c>
       <c r="H40" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
       <c r="A41" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B41" t="s">
+        <v>113</v>
+      </c>
+      <c r="C41" t="s">
         <v>114</v>
       </c>
-      <c r="C41" t="s">
-        <v>115</v>
-      </c>
       <c r="D41" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E41">
         <v>4</v>
@@ -2274,7 +2271,7 @@
         <v>21</v>
       </c>
       <c r="H41" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -2291,16 +2288,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A7EA96D-7C78-2A4B-AAB8-1FB20EF8C6D6}">
   <dimension ref="A1:I49"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
   <cols>
     <col min="1" max="1" width="16.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="27.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="35.5" customWidth="1"/>
-    <col min="8" max="8" width="73.6640625" customWidth="1"/>
+    <col min="8" max="8" width="73.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" s="3" customFormat="1">
       <c r="A1" s="3" t="s">
         <v>7</v>
       </c>
@@ -2326,44 +2323,44 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" t="s">
         <v>64</v>
       </c>
-      <c r="C2" t="s">
-        <v>65</v>
-      </c>
       <c r="D2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E2">
         <v>0.86</v>
       </c>
       <c r="F2" t="s">
+        <v>116</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" t="s">
         <v>117</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" t="s">
         <v>61</v>
       </c>
-      <c r="C3" t="s">
-        <v>62</v>
-      </c>
       <c r="D3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E3">
         <v>0.96</v>
@@ -2375,21 +2372,21 @@
         <v>21</v>
       </c>
       <c r="H3" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" t="s">
         <v>48</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>49</v>
       </c>
-      <c r="C4" t="s">
-        <v>50</v>
-      </c>
       <c r="D4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E4">
         <v>0.85</v>
@@ -2401,21 +2398,21 @@
         <v>21</v>
       </c>
       <c r="H4" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5" t="s">
         <v>58</v>
       </c>
-      <c r="C5" t="s">
-        <v>59</v>
-      </c>
       <c r="D5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E5">
         <v>0.81</v>
@@ -2427,21 +2424,21 @@
         <v>21</v>
       </c>
       <c r="H5" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" t="s">
         <v>55</v>
       </c>
-      <c r="C6" t="s">
-        <v>56</v>
-      </c>
       <c r="D6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E6">
         <v>0.92</v>
@@ -2453,21 +2450,21 @@
         <v>21</v>
       </c>
       <c r="H6" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" t="s">
         <v>52</v>
       </c>
-      <c r="C7" t="s">
-        <v>53</v>
-      </c>
       <c r="D7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E7">
         <v>0.7</v>
@@ -2479,21 +2476,21 @@
         <v>21</v>
       </c>
       <c r="H7" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
       <c r="A8" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B8" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>109</v>
-      </c>
       <c r="D8" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E8" s="5">
         <v>0.97</v>
@@ -2505,22 +2502,22 @@
         <v>21</v>
       </c>
       <c r="H8" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="I8" s="6"/>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>124</v>
-      </c>
-      <c r="I8" s="6"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A9" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>125</v>
       </c>
       <c r="E9" s="5">
         <v>0.8</v>
@@ -2532,22 +2529,22 @@
         <v>21</v>
       </c>
       <c r="H9" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I9" s="6"/>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>126</v>
-      </c>
-      <c r="I9" s="6"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A10" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>127</v>
       </c>
       <c r="E10" s="5">
         <v>2</v>
@@ -2559,22 +2556,22 @@
         <v>21</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I10" s="6"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9">
       <c r="A11" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="C11" s="5" t="s">
-        <v>105</v>
-      </c>
       <c r="D11" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E11" s="5">
         <v>0.97</v>
@@ -2586,22 +2583,22 @@
         <v>21</v>
       </c>
       <c r="H11" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="I11" s="6"/>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D12" s="5" t="s">
         <v>124</v>
-      </c>
-      <c r="I11" s="6"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>125</v>
       </c>
       <c r="E12" s="5">
         <v>0.9</v>
@@ -2613,22 +2610,22 @@
         <v>21</v>
       </c>
       <c r="H12" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I12" s="6"/>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>126</v>
-      </c>
-      <c r="I12" s="6"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>127</v>
       </c>
       <c r="E13" s="5">
         <v>1</v>
@@ -2640,22 +2637,22 @@
         <v>21</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I13" s="6"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9">
       <c r="A14" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B14" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>115</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>116</v>
       </c>
       <c r="E14" s="5">
         <v>0.99</v>
@@ -2667,22 +2664,22 @@
         <v>21</v>
       </c>
       <c r="H14" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="I14" s="6"/>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="D15" s="5" t="s">
         <v>124</v>
-      </c>
-      <c r="I14" s="6"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A15" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>125</v>
       </c>
       <c r="E15" s="5">
         <v>0.97</v>
@@ -2694,22 +2691,22 @@
         <v>21</v>
       </c>
       <c r="H15" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I15" s="6"/>
+    </row>
+    <row r="16" spans="1:9" ht="84.95">
+      <c r="A16" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="D16" s="5" t="s">
         <v>126</v>
-      </c>
-      <c r="I15" s="6"/>
-    </row>
-    <row r="16" spans="1:9" ht="85" x14ac:dyDescent="0.2">
-      <c r="A16" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>127</v>
       </c>
       <c r="E16" s="5">
         <v>1</v>
@@ -2721,24 +2718,24 @@
         <v>21</v>
       </c>
       <c r="H16" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="I16" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="I16" s="7" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="17" spans="1:9">
       <c r="A17" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B17" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="C17" s="5" t="s">
-        <v>101</v>
-      </c>
       <c r="D17" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E17" s="5">
         <v>0.99</v>
@@ -2750,22 +2747,22 @@
         <v>21</v>
       </c>
       <c r="H17" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="I17" s="6"/>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>124</v>
-      </c>
-      <c r="I17" s="6"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A18" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>125</v>
       </c>
       <c r="E18" s="5">
         <v>0.97</v>
@@ -2777,22 +2774,22 @@
         <v>21</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I18" s="6"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9">
       <c r="A19" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B19" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="C19" s="5" t="s">
-        <v>101</v>
-      </c>
       <c r="D19" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E19" s="5">
         <v>1</v>
@@ -2804,22 +2801,22 @@
         <v>21</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I19" s="6"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9">
       <c r="A20" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B20" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="C20" s="5" t="s">
-        <v>111</v>
-      </c>
       <c r="D20" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E20" s="5">
         <v>0.99</v>
@@ -2831,22 +2828,22 @@
         <v>21</v>
       </c>
       <c r="H20" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="I20" s="6"/>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="D21" s="5" t="s">
         <v>124</v>
-      </c>
-      <c r="I20" s="6"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A21" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>125</v>
       </c>
       <c r="E21" s="5">
         <v>0.97</v>
@@ -2858,22 +2855,22 @@
         <v>21</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I21" s="6"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:9">
       <c r="A22" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B22" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C22" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="C22" s="5" t="s">
-        <v>111</v>
-      </c>
       <c r="D22" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E22" s="5">
         <v>1.5</v>
@@ -2885,22 +2882,22 @@
         <v>21</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I22" s="6"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9">
       <c r="A23" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B23" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="C23" s="5" t="s">
-        <v>95</v>
-      </c>
       <c r="D23" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E23" s="5">
         <v>0.97</v>
@@ -2912,22 +2909,22 @@
         <v>21</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I23" s="6"/>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:9">
       <c r="A24" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B24" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C24" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="C24" s="5" t="s">
-        <v>95</v>
-      </c>
       <c r="D24" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E24" s="5">
         <v>0.7</v>
@@ -2939,22 +2936,22 @@
         <v>21</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I24" s="6"/>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:9">
       <c r="A25" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B25" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C25" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="C25" s="5" t="s">
-        <v>95</v>
-      </c>
       <c r="D25" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E25" s="5">
         <v>1</v>
@@ -2966,22 +2963,22 @@
         <v>21</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I25" s="6"/>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:9">
       <c r="A26" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B26" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C26" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="C26" s="5" t="s">
-        <v>91</v>
-      </c>
       <c r="D26" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E26" s="5">
         <v>0.97</v>
@@ -2993,22 +2990,22 @@
         <v>21</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I26" s="6"/>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:9">
       <c r="A27" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B27" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C27" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="C27" s="5" t="s">
-        <v>91</v>
-      </c>
       <c r="D27" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E27" s="5">
         <v>0.7</v>
@@ -3020,22 +3017,22 @@
         <v>21</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I27" s="6"/>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:9">
       <c r="A28" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B28" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C28" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="C28" s="5" t="s">
-        <v>91</v>
-      </c>
       <c r="D28" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E28" s="5">
         <v>1</v>
@@ -3047,22 +3044,22 @@
         <v>21</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I28" s="6"/>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:9">
       <c r="A29" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B29" t="s">
+        <v>85</v>
+      </c>
+      <c r="C29" t="s">
         <v>86</v>
       </c>
-      <c r="C29" t="s">
-        <v>87</v>
-      </c>
       <c r="D29" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E29">
         <v>0.98</v>
@@ -3074,21 +3071,21 @@
         <v>21</v>
       </c>
       <c r="H29" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B30" t="s">
+        <v>85</v>
+      </c>
+      <c r="C30" t="s">
         <v>86</v>
       </c>
-      <c r="C30" t="s">
-        <v>87</v>
-      </c>
       <c r="D30" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E30">
         <v>0.95</v>
@@ -3100,21 +3097,21 @@
         <v>21</v>
       </c>
       <c r="H30" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9">
       <c r="A31" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B31" t="s">
+        <v>85</v>
+      </c>
+      <c r="C31" t="s">
         <v>86</v>
       </c>
-      <c r="C31" t="s">
-        <v>87</v>
-      </c>
       <c r="D31" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -3126,21 +3123,21 @@
         <v>21</v>
       </c>
       <c r="H31" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9">
       <c r="A32" t="s">
+        <v>79</v>
+      </c>
+      <c r="B32" t="s">
         <v>80</v>
       </c>
-      <c r="B32" t="s">
+      <c r="C32" t="s">
         <v>81</v>
       </c>
-      <c r="C32" t="s">
-        <v>82</v>
-      </c>
       <c r="D32" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E32">
         <v>0.99</v>
@@ -3152,21 +3149,21 @@
         <v>21</v>
       </c>
       <c r="H32" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
       <c r="A33" t="s">
+        <v>79</v>
+      </c>
+      <c r="B33" t="s">
         <v>80</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
         <v>81</v>
       </c>
-      <c r="C33" t="s">
-        <v>82</v>
-      </c>
       <c r="D33" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E33">
         <v>0.97</v>
@@ -3178,21 +3175,21 @@
         <v>21</v>
       </c>
       <c r="H33" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
       <c r="A34" t="s">
+        <v>79</v>
+      </c>
+      <c r="B34" t="s">
         <v>80</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
         <v>81</v>
       </c>
-      <c r="C34" t="s">
-        <v>82</v>
-      </c>
       <c r="D34" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E34">
         <v>1</v>
@@ -3204,21 +3201,21 @@
         <v>21</v>
       </c>
       <c r="H34" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
       <c r="A35" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B35" t="s">
+        <v>95</v>
+      </c>
+      <c r="C35" t="s">
         <v>96</v>
       </c>
-      <c r="C35" t="s">
-        <v>97</v>
-      </c>
       <c r="D35" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E35">
         <v>0.99</v>
@@ -3230,21 +3227,21 @@
         <v>21</v>
       </c>
       <c r="H35" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
       <c r="A36" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B36" t="s">
+        <v>95</v>
+      </c>
+      <c r="C36" t="s">
         <v>96</v>
       </c>
-      <c r="C36" t="s">
-        <v>97</v>
-      </c>
       <c r="D36" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E36">
         <v>0.97</v>
@@ -3256,21 +3253,21 @@
         <v>21</v>
       </c>
       <c r="H36" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
       <c r="A37" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B37" t="s">
+        <v>95</v>
+      </c>
+      <c r="C37" t="s">
         <v>96</v>
       </c>
-      <c r="C37" t="s">
-        <v>97</v>
-      </c>
       <c r="D37" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E37">
         <v>1</v>
@@ -3282,47 +3279,47 @@
         <v>21</v>
       </c>
       <c r="H37" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
       <c r="A38" t="s">
         <v>26</v>
       </c>
       <c r="B38" t="s">
+        <v>44</v>
+      </c>
+      <c r="C38" t="s">
         <v>45</v>
       </c>
-      <c r="C38" t="s">
-        <v>46</v>
-      </c>
       <c r="D38" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E38">
         <v>0.3</v>
       </c>
       <c r="F38" t="s">
+        <v>140</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H38" t="s">
         <v>141</v>
       </c>
-      <c r="G38" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H38" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="39" spans="1:8">
       <c r="A39" t="s">
         <v>26</v>
       </c>
       <c r="B39" t="s">
+        <v>41</v>
+      </c>
+      <c r="C39" t="s">
         <v>42</v>
       </c>
-      <c r="C39" t="s">
-        <v>43</v>
-      </c>
       <c r="D39" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E39">
         <v>0.75</v>
@@ -3334,10 +3331,10 @@
         <v>21</v>
       </c>
       <c r="H39" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
       <c r="A40" t="s">
         <v>26</v>
       </c>
@@ -3348,7 +3345,7 @@
         <v>31</v>
       </c>
       <c r="D40" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E40">
         <v>0.88</v>
@@ -3360,10 +3357,10 @@
         <v>21</v>
       </c>
       <c r="H40" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
       <c r="A41" t="s">
         <v>26</v>
       </c>
@@ -3374,7 +3371,7 @@
         <v>33</v>
       </c>
       <c r="D41" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E41">
         <v>0.92</v>
@@ -3386,10 +3383,10 @@
         <v>21</v>
       </c>
       <c r="H41" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
       <c r="A42" t="s">
         <v>26</v>
       </c>
@@ -3400,7 +3397,7 @@
         <v>28</v>
       </c>
       <c r="D42" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E42">
         <v>0.95</v>
@@ -3412,21 +3409,21 @@
         <v>21</v>
       </c>
       <c r="H42" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
       <c r="A43" t="s">
+        <v>69</v>
+      </c>
+      <c r="B43" t="s">
         <v>70</v>
       </c>
-      <c r="B43" t="s">
+      <c r="C43" t="s">
         <v>71</v>
       </c>
-      <c r="C43" t="s">
-        <v>72</v>
-      </c>
       <c r="D43" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E43">
         <v>0.8</v>
@@ -3438,21 +3435,21 @@
         <v>21</v>
       </c>
       <c r="H43" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
       <c r="A44" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B44" t="s">
+        <v>76</v>
+      </c>
+      <c r="C44" t="s">
         <v>77</v>
       </c>
-      <c r="C44" t="s">
-        <v>78</v>
-      </c>
       <c r="D44" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E44">
         <v>0.3</v>
@@ -3464,21 +3461,21 @@
         <v>21</v>
       </c>
       <c r="H44" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
       <c r="A45" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B45" t="s">
+        <v>73</v>
+      </c>
+      <c r="C45" t="s">
         <v>74</v>
       </c>
-      <c r="C45" t="s">
-        <v>75</v>
-      </c>
       <c r="D45" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E45">
         <v>0.88</v>
@@ -3490,10 +3487,10 @@
         <v>21</v>
       </c>
       <c r="H45" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8">
       <c r="A46" t="s">
         <v>16</v>
       </c>
@@ -3504,7 +3501,7 @@
         <v>24</v>
       </c>
       <c r="D46" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E46">
         <v>1</v>
@@ -3516,7 +3513,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:8">
       <c r="A47" t="s">
         <v>16</v>
       </c>
@@ -3527,7 +3524,7 @@
         <v>18</v>
       </c>
       <c r="D47" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E47">
         <v>0.85</v>
@@ -3539,21 +3536,21 @@
         <v>21</v>
       </c>
       <c r="H47" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
       <c r="A48" t="s">
         <v>26</v>
       </c>
       <c r="B48" t="s">
+        <v>34</v>
+      </c>
+      <c r="C48" t="s">
         <v>35</v>
       </c>
-      <c r="C48" t="s">
-        <v>36</v>
-      </c>
       <c r="D48" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E48">
         <v>0.15</v>
@@ -3565,21 +3562,21 @@
         <v>21</v>
       </c>
       <c r="H48" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
       <c r="A49" t="s">
         <v>26</v>
       </c>
       <c r="B49" t="s">
+        <v>36</v>
+      </c>
+      <c r="C49" t="s">
         <v>37</v>
       </c>
-      <c r="C49" t="s">
-        <v>38</v>
-      </c>
       <c r="D49" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E49">
         <v>0.15</v>
@@ -3591,7 +3588,7 @@
         <v>21</v>
       </c>
       <c r="H49" t="s">
-        <v>201</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -3602,385 +3599,385 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6747B679-9230-3847-955E-AE6563A4F4F1}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
   <cols>
     <col min="1" max="1" width="30" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="42.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="106.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="106.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" s="3" customFormat="1">
       <c r="A1" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B2">
         <v>0.02</v>
       </c>
       <c r="C2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D2" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="E2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F2" t="s">
+        <v>160</v>
+      </c>
+      <c r="G2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>162</v>
+      </c>
+      <c r="B3" t="s">
+        <v>163</v>
+      </c>
+      <c r="C3" t="s">
         <v>158</v>
       </c>
-      <c r="E2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="D3" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="G2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>161</v>
-      </c>
-      <c r="B3" t="s">
-        <v>162</v>
-      </c>
-      <c r="C3" t="s">
-        <v>157</v>
-      </c>
-      <c r="D3" s="8" t="s">
+      <c r="E3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F3" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>165</v>
+      </c>
+      <c r="B4" t="s">
+        <v>163</v>
+      </c>
+      <c r="C4" t="s">
         <v>158</v>
       </c>
-      <c r="E3" t="s">
-        <v>41</v>
-      </c>
-      <c r="F3" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>164</v>
-      </c>
-      <c r="B4" t="s">
-        <v>162</v>
-      </c>
-      <c r="C4" t="s">
-        <v>157</v>
-      </c>
       <c r="D4" s="8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F4" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B5">
         <v>1.5</v>
       </c>
       <c r="C5" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F5" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B6">
         <v>0.6</v>
       </c>
       <c r="C6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F6" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B7">
         <v>0.85</v>
       </c>
       <c r="C7" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F7" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B8">
         <v>0.08</v>
       </c>
       <c r="C8" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F8" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B9">
         <v>0.15</v>
       </c>
       <c r="C9" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F9" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B10">
         <v>0.05</v>
       </c>
       <c r="C10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F10" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B11">
         <v>0.25</v>
       </c>
       <c r="C11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E11" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F11" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B12">
         <v>0.02</v>
       </c>
       <c r="C12" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F12" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B13">
         <v>0.2</v>
       </c>
       <c r="C13" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F13" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B14">
         <v>0.9</v>
       </c>
       <c r="C14" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F14" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B15">
         <v>0.9</v>
       </c>
       <c r="C15" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E15" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F15" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B16">
         <v>0.1</v>
       </c>
       <c r="C16" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F16" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B17">
         <v>0.5</v>
       </c>
       <c r="C17" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E17" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F17" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
       <c r="A18" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B18" s="1">
         <v>0.9</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>21</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B19">
         <v>0.15</v>
@@ -3992,15 +3989,15 @@
         <v>21</v>
       </c>
       <c r="E19" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F19" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B20">
         <v>0.3</v>
@@ -4012,10 +4009,10 @@
         <v>21</v>
       </c>
       <c r="E20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F20" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
First infections and prevention
</commit_message>
<xml_diff>
--- a/data/TierPlus Parameter Lists - Shared.xlsx
+++ b/data/TierPlus Parameter Lists - Shared.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="256" documentId="8_{3B20D403-37D7-C947-81A8-DEC9FA14756B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA5ECF80-BE53-2D41-8922-3136AC45F1AA}"/>
+  <xr:revisionPtr revIDLastSave="275" documentId="8_{3B20D403-37D7-C947-81A8-DEC9FA14756B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4CB68141-40CA-A248-938A-C3818F399AB5}"/>
   <bookViews>
-    <workbookView xWindow="-2380" yWindow="-18780" windowWidth="27020" windowHeight="15820" activeTab="3" xr2:uid="{3655CBE5-0E8F-BC41-8085-555297440F15}"/>
+    <workbookView xWindow="5440" yWindow="-19220" windowWidth="27020" windowHeight="15820" activeTab="3" xr2:uid="{3655CBE5-0E8F-BC41-8085-555297440F15}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="7" r:id="rId1"/>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="769" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="783" uniqueCount="214">
   <si>
     <t>Values need to incoporate realistic implementation and weighted effects</t>
   </si>
@@ -580,9 +580,6 @@
     <t>hiv_mortality_on_treatment</t>
   </si>
   <si>
-    <t>0.098 (up to 0.63 for AIDS stage... calibration?)</t>
-  </si>
-  <si>
     <t>HIV related mortality while on tretament but not virally suppressed</t>
   </si>
   <si>
@@ -613,9 +610,6 @@
     <t>ltfu_rate</t>
   </si>
   <si>
-    <t>annual rate of LTFU</t>
-  </si>
-  <si>
     <t>high_risk_proprtion</t>
   </si>
   <si>
@@ -719,6 +713,27 @@
   </si>
   <si>
     <t>HIV related mortality first year on treatment non AHD</t>
+  </si>
+  <si>
+    <t>ltfu_suppressed</t>
+  </si>
+  <si>
+    <t>ltfu_unsuppressed</t>
+  </si>
+  <si>
+    <t>starting population of LTFU</t>
+  </si>
+  <si>
+    <t>Annual LTFU rate among those suppressed</t>
+  </si>
+  <si>
+    <t>Annual LTFU rate among those unsuppressed</t>
+  </si>
+  <si>
+    <t>retention_intervention_suppression</t>
+  </si>
+  <si>
+    <t>Rate of viral suppression among those kept in care by retention interventions</t>
   </si>
 </sst>
 </file>
@@ -1400,7 +1415,7 @@
         <v>34</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="D7" t="s">
         <v>19</v>
@@ -1426,7 +1441,7 @@
         <v>36</v>
       </c>
       <c r="C8" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D8" t="s">
         <v>19</v>
@@ -3445,10 +3460,10 @@
         <v>26</v>
       </c>
       <c r="B43" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="D43" t="s">
         <v>115</v>
@@ -3471,10 +3486,10 @@
         <v>26</v>
       </c>
       <c r="B44" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C44" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D44" t="s">
         <v>115</v>
@@ -3678,7 +3693,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6747B679-9230-3847-955E-AE6563A4F4F1}">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" bestFit="1" customWidth="1"/>
@@ -3714,7 +3729,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B2">
         <v>9.8000000000000004E-2</v>
@@ -3729,7 +3744,7 @@
         <v>40</v>
       </c>
       <c r="F2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="G2" t="s">
         <v>160</v>
@@ -3739,8 +3754,8 @@
       <c r="A3" t="s">
         <v>161</v>
       </c>
-      <c r="B3" t="s">
-        <v>162</v>
+      <c r="B3">
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="C3" t="s">
         <v>158</v>
@@ -3752,7 +3767,7 @@
         <v>40</v>
       </c>
       <c r="F3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G3" t="s">
         <v>159</v>
@@ -3762,8 +3777,8 @@
       <c r="A4" t="s">
         <v>157</v>
       </c>
-      <c r="B4" t="s">
-        <v>162</v>
+      <c r="B4">
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="C4" t="s">
         <v>158</v>
@@ -3775,12 +3790,12 @@
         <v>40</v>
       </c>
       <c r="F4" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B5">
         <v>0.2</v>
@@ -3795,15 +3810,18 @@
         <v>40</v>
       </c>
       <c r="F5" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B6">
-        <v>0.02</v>
+        <v>0.06</v>
+      </c>
+      <c r="C6" t="s">
+        <v>158</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>21</v>
@@ -3812,12 +3830,12 @@
         <v>40</v>
       </c>
       <c r="F6" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B7">
         <v>1.5</v>
@@ -3832,12 +3850,12 @@
         <v>40</v>
       </c>
       <c r="F7" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B8">
         <v>0.6</v>
@@ -3852,12 +3870,12 @@
         <v>40</v>
       </c>
       <c r="F8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B9">
         <v>0.85</v>
@@ -3872,12 +3890,12 @@
         <v>40</v>
       </c>
       <c r="F9" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B10">
         <v>0.08</v>
@@ -3892,12 +3910,12 @@
         <v>40</v>
       </c>
       <c r="F10" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B11">
         <v>0.15</v>
@@ -3912,12 +3930,12 @@
         <v>40</v>
       </c>
       <c r="F11" t="s">
-        <v>173</v>
+        <v>209</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B12">
         <v>0.05</v>
@@ -3932,12 +3950,12 @@
         <v>40</v>
       </c>
       <c r="F12" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B13">
         <v>0.25</v>
@@ -3949,15 +3967,15 @@
         <v>21</v>
       </c>
       <c r="E13" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="F13" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B14">
         <v>0.02</v>
@@ -3972,12 +3990,12 @@
         <v>40</v>
       </c>
       <c r="F14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B15">
         <v>0.2</v>
@@ -3992,15 +4010,15 @@
         <v>40</v>
       </c>
       <c r="F15" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B16">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="C16" t="s">
         <v>158</v>
@@ -4012,15 +4030,15 @@
         <v>40</v>
       </c>
       <c r="F16" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B17">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="C17" t="s">
         <v>158</v>
@@ -4032,12 +4050,12 @@
         <v>40</v>
       </c>
       <c r="F17" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B18">
         <v>0.1</v>
@@ -4052,12 +4070,12 @@
         <v>40</v>
       </c>
       <c r="F18" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B19">
         <v>0.5</v>
@@ -4069,15 +4087,15 @@
         <v>21</v>
       </c>
       <c r="E19" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="F19" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B20" s="1">
         <v>0.9</v>
@@ -4089,15 +4107,15 @@
         <v>21</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B21">
         <v>0.15</v>
@@ -4109,15 +4127,15 @@
         <v>21</v>
       </c>
       <c r="E21" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="F21" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B22">
         <v>0.3</v>
@@ -4132,7 +4150,67 @@
         <v>40</v>
       </c>
       <c r="F22" t="s">
-        <v>197</v>
+        <v>195</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>207</v>
+      </c>
+      <c r="B23">
+        <v>0.05</v>
+      </c>
+      <c r="C23" t="s">
+        <v>20</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E23" t="s">
+        <v>40</v>
+      </c>
+      <c r="F23" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>208</v>
+      </c>
+      <c r="B24">
+        <v>0.15</v>
+      </c>
+      <c r="C24" t="s">
+        <v>20</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E24" t="s">
+        <v>40</v>
+      </c>
+      <c r="F24" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>212</v>
+      </c>
+      <c r="B25">
+        <v>0.3</v>
+      </c>
+      <c r="C25" t="s">
+        <v>20</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E25" t="s">
+        <v>40</v>
+      </c>
+      <c r="F25" t="s">
+        <v>213</v>
       </c>
     </row>
   </sheetData>

</xml_diff>